<commit_message>
Add office and block codes; show only PINs during randomisation
- Officers: Office Code, Home Block Code, Posting Block Code; booths: Block Code
- Codes decide "same office" and "same block" when present, so spelling
  mistakes in names no longer split one office/block into two; names are
  used only where a code is missing
- Warnings for one name with two codes and one code with two spellings
- 2nd and final randomisation screens and the shuffle animation show PINs
  only; letters, reports, attendance sheets and exports keep full details
- Templates, test data, project Excel and tests updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V5zeq2JHM1LeQHsBokCXrg
</commit_message>
<xml_diff>
--- a/test-data/Booths_Template.xlsx
+++ b/test-data/Booths_Template.xlsx
@@ -398,13 +398,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F4"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
     <col min="3" max="3" width="10.83203125" customWidth="1"/>
     <col min="4" max="4" width="44.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -421,6 +422,9 @@
         <v>Location / Building</v>
       </c>
       <c r="E1" t="str">
+        <v>Block Code</v>
+      </c>
+      <c r="F1" t="str">
         <v>Block</v>
       </c>
     </row>
@@ -438,6 +442,9 @@
         <v>Upgraded High School, Room 1</v>
       </c>
       <c r="E2" t="str">
+        <v>0102</v>
+      </c>
+      <c r="F2" t="str">
         <v>Piprahi</v>
       </c>
     </row>
@@ -455,6 +462,9 @@
         <v>Upgraded High School, Room 2</v>
       </c>
       <c r="E3" t="str">
+        <v>0102</v>
+      </c>
+      <c r="F3" t="str">
         <v>Piprahi</v>
       </c>
     </row>
@@ -472,19 +482,22 @@
         <v>Block Office Hall</v>
       </c>
       <c r="E4" t="str">
+        <v>0105</v>
+      </c>
+      <c r="F4" t="str">
         <v>Tariyani</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A5"/>
   <cols>
     <col min="1" max="1" width="120.83203125" customWidth="1"/>
   </cols>
@@ -506,12 +519,17 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
+        <v>Block Code (e.g. census block code) is recommended: when the booth and the officer both have a code, the code decides and spelling of the name does not matter.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
         <v>Delete the example rows before use.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix Aux booth type lost on Excel import; fuller template instructions
- Booth rows imported from Excel (template or project file) always came
  in as "Main" because the default value blocked the sheet value. Aux is
  now kept; test covers save/open of 19 Aux booths.
- Officer and booth templates: field-by-field instructions, an
  out-of-district (999999 / Others) example row, note on leading zeros.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V5zeq2JHM1LeQHsBokCXrg
</commit_message>
<xml_diff>
--- a/test-data/Booths_Template.xlsx
+++ b/test-data/Booths_Template.xlsx
@@ -497,39 +497,59 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A9"/>
   <cols>
     <col min="1" max="1" width="120.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Constituency = a code from Setup (TC, GC).</v>
+        <v>BOOTHS — one row per polling station. Delete the example rows before use.</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Main/Aux = Main or Aux.</v>
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Block is mandatory — officers whose home or posting block is this block are never tagged to this booth.</v>
+        <v>Constituency        — a code from Setup (TC, GC), or a name containing "Teachers" / "Graduates".</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Block Code (e.g. census block code) is recommended: when the booth and the officer both have a code, the code decides and spelling of the name does not matter.</v>
+        <v>Booth No            — e.g. 12 or 12A; unique within the constituency.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Delete the example rows before use.</v>
+        <v>Main/Aux            — Main or Aux.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Location / Building — printed on the final letter.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Block Code / Block  — mandatory (name or code). Officers whose home or posting block is this block are never tagged to this booth.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v xml:space="preserve">                      Block Code (e.g. 2011 census code) is recommended — it must be the same code used in the Officers sheet.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v xml:space="preserve">                      A booth must never use the out-of-district code 999999 / "Others".</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>